<commit_message>
New CHanges and Formatting
</commit_message>
<xml_diff>
--- a/Machine Learning/PII/Interim-report/Papers/Papers-Table.xlsx
+++ b/Machine Learning/PII/Interim-report/Papers/Papers-Table.xlsx
@@ -1,23 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\git\Machine Learning\PII\Interim-report\Papers\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B4E3103-B6E0-424D-A661-677C7101B382}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FACFA10-53CF-4D9E-B65C-36175A7F2838}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{AA821531-E608-40CF-B71D-4D7770E4DFA0}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{AA821531-E608-40CF-B71D-4D7770E4DFA0}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="LLM Questions" sheetId="2" r:id="rId2"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$K$1</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -4121,7 +4123,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -4179,12 +4181,6 @@
     </font>
     <font>
       <i/>
-      <sz val="8"/>
-      <color rgb="FF47484C"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
       <sz val="8"/>
       <color rgb="FF47484C"/>
       <name val="Arial"/>
@@ -4570,20 +4566,20 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E3273017-25D8-4705-B64D-E4EEBFC32101}">
   <dimension ref="A1:K29"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="28.21875" style="2" customWidth="1"/>
-    <col min="3" max="3" width="12.33203125" style="2" customWidth="1"/>
-    <col min="4" max="4" width="7.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.85546875" style="2" customWidth="1"/>
+    <col min="3" max="3" width="12.28515625" style="2" customWidth="1"/>
+    <col min="4" max="4" width="7.28515625" customWidth="1"/>
     <col min="5" max="5" width="42" style="2" customWidth="1"/>
-    <col min="6" max="6" width="39.44140625" customWidth="1"/>
-    <col min="7" max="7" width="32.77734375" style="2" customWidth="1"/>
-    <col min="8" max="8" width="33.44140625" style="2" customWidth="1"/>
-    <col min="9" max="9" width="29.33203125" customWidth="1"/>
-    <col min="10" max="10" width="40.77734375" customWidth="1"/>
+    <col min="6" max="6" width="12" customWidth="1"/>
+    <col min="7" max="7" width="17.140625" style="2" customWidth="1"/>
+    <col min="8" max="8" width="17.7109375" style="2" customWidth="1"/>
+    <col min="9" max="9" width="11" customWidth="1"/>
+    <col min="10" max="10" width="40.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" s="7" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
         <v>26</v>
       </c>
@@ -4618,7 +4614,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="154.19999999999999" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:11" ht="180.75" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -4644,795 +4640,808 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="215.4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:11" ht="409.6" x14ac:dyDescent="0.25">
       <c r="A3">
+        <v>4</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C3" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="D3" s="1">
+        <v>45778</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" ht="409.6" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>14</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="C4" s="9" t="s">
+        <v>99</v>
+      </c>
+      <c r="D4" s="1">
+        <v>45748</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>17</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="C5" s="9" t="s">
+        <v>123</v>
+      </c>
+      <c r="D5" s="1">
+        <v>45748</v>
+      </c>
+      <c r="E5" s="11" t="s">
+        <v>124</v>
+      </c>
+      <c r="F5" s="11" t="s">
+        <v>125</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="I5" s="2" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" ht="409.6" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>7</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="C6" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="D6" s="1">
+        <v>45505</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="I6" s="2" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A7" s="12">
+        <v>19</v>
+      </c>
+      <c r="B7" s="16" t="s">
+        <v>137</v>
+      </c>
+      <c r="C7" s="13" t="s">
+        <v>138</v>
+      </c>
+      <c r="D7" s="14">
+        <v>45505</v>
+      </c>
+      <c r="E7" s="15" t="s">
+        <v>139</v>
+      </c>
+      <c r="F7" s="16" t="s">
+        <v>140</v>
+      </c>
+      <c r="G7" s="16" t="s">
+        <v>141</v>
+      </c>
+      <c r="H7" s="16" t="s">
+        <v>142</v>
+      </c>
+      <c r="I7" s="16" t="s">
+        <v>143</v>
+      </c>
+      <c r="J7" s="12"/>
+      <c r="K7" s="12"/>
+    </row>
+    <row r="8" spans="1:11" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>21</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="C8" s="9" t="s">
+        <v>152</v>
+      </c>
+      <c r="D8" s="1">
+        <v>45383</v>
+      </c>
+      <c r="E8" s="11" t="s">
+        <v>153</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="I8" s="2" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>20</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="D9" s="1">
+        <v>45352</v>
+      </c>
+      <c r="E9" s="11" t="s">
+        <v>146</v>
+      </c>
+      <c r="F9" s="11" t="s">
+        <v>147</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="I9" s="2" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>28</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="C10" s="9" t="s">
+        <v>201</v>
+      </c>
+      <c r="D10" s="1">
+        <v>45292</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>204</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>205</v>
+      </c>
+      <c r="H10" s="2" t="s">
+        <v>206</v>
+      </c>
+      <c r="I10" s="2" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>22</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="C11" s="9" t="s">
+        <v>159</v>
+      </c>
+      <c r="D11" s="1">
+        <v>45261</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="G11" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="H11" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="I11" s="2" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" ht="409.6" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>3</v>
+      </c>
+      <c r="B12" t="s">
+        <v>20</v>
+      </c>
+      <c r="C12"/>
+      <c r="D12" s="1">
+        <v>45170</v>
+      </c>
+      <c r="E12" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="F12" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="G12" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="H12" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="I12" s="2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" ht="409.6" x14ac:dyDescent="0.25">
+      <c r="A13">
         <v>2</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B13" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="D3" s="1">
+      <c r="D13" s="1">
         <v>45121</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="E13" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="F3" s="4" t="s">
+      <c r="F13" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="G3" s="3" t="s">
+      <c r="G13" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="H3" s="3" t="s">
+      <c r="H13" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="I3" s="3" t="s">
+      <c r="I13" s="3" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="256.2" x14ac:dyDescent="0.3">
-      <c r="A4">
-        <v>3</v>
-      </c>
-      <c r="B4" t="s">
-        <v>20</v>
-      </c>
-      <c r="C4"/>
-      <c r="D4" s="1">
-        <v>45170</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="F4" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="G4" s="4" t="s">
+    <row r="14" spans="1:11" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A14" s="12">
+        <v>15</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="C14" s="13" t="s">
+        <v>107</v>
+      </c>
+      <c r="D14" s="14">
+        <v>45078</v>
+      </c>
+      <c r="E14" s="15" t="s">
+        <v>108</v>
+      </c>
+      <c r="F14" s="16" t="s">
+        <v>109</v>
+      </c>
+      <c r="G14" s="16" t="s">
+        <v>110</v>
+      </c>
+      <c r="H14" s="16" t="s">
+        <v>111</v>
+      </c>
+      <c r="I14" s="16" t="s">
+        <v>114</v>
+      </c>
+      <c r="J14" s="16" t="s">
+        <v>112</v>
+      </c>
+      <c r="K14" s="12"/>
+    </row>
+    <row r="15" spans="1:11" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>23</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="C15" s="9" t="s">
+        <v>165</v>
+      </c>
+      <c r="D15" s="1">
+        <v>45078</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="G15" s="2" t="s">
+        <v>169</v>
+      </c>
+      <c r="H15" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="I15" s="2" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" s="12" customFormat="1" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>6</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C16" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="D16" s="10">
+        <v>45047</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="G16" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="H16" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="I16" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="J16" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="K16"/>
+    </row>
+    <row r="17" spans="1:11" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>18</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="C17" s="9" t="s">
+        <v>131</v>
+      </c>
+      <c r="D17" s="1">
+        <v>45047</v>
+      </c>
+      <c r="E17" s="11" t="s">
+        <v>132</v>
+      </c>
+      <c r="F17" s="11" t="s">
+        <v>133</v>
+      </c>
+      <c r="G17" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="H17" s="11" t="s">
+        <v>135</v>
+      </c>
+      <c r="I17" s="11" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A18">
         <v>24</v>
       </c>
-      <c r="H4" s="4" t="s">
+      <c r="B18" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="C18" s="9" t="s">
+        <v>172</v>
+      </c>
+      <c r="D18" s="1">
+        <v>44958</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="F18" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="G18" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="H18" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="I18" s="2" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A19">
+        <v>13</v>
+      </c>
+      <c r="B19" t="s">
+        <v>92</v>
+      </c>
+      <c r="C19" s="9" t="s">
+        <v>93</v>
+      </c>
+      <c r="D19" s="1">
+        <v>44743</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="F19" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="G19" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="H19" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="I19" s="2" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" s="12" customFormat="1" ht="409.6" x14ac:dyDescent="0.25">
+      <c r="A20">
+        <v>16</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="C20" s="9" t="s">
+        <v>116</v>
+      </c>
+      <c r="D20" s="1">
+        <v>44593</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="F20" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="G20" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="H20" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="I20" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="J20"/>
+      <c r="K20"/>
+    </row>
+    <row r="21" spans="1:11" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A21" s="12">
+        <v>27</v>
+      </c>
+      <c r="B21" s="16" t="s">
+        <v>195</v>
+      </c>
+      <c r="C21" s="13" t="s">
+        <v>93</v>
+      </c>
+      <c r="D21" s="14">
+        <v>44470</v>
+      </c>
+      <c r="E21" s="16" t="s">
+        <v>196</v>
+      </c>
+      <c r="F21" s="16" t="s">
+        <v>197</v>
+      </c>
+      <c r="G21" s="16" t="s">
+        <v>198</v>
+      </c>
+      <c r="H21" s="16" t="s">
+        <v>199</v>
+      </c>
+      <c r="I21" s="16" t="s">
+        <v>200</v>
+      </c>
+      <c r="J21" s="12"/>
+      <c r="K21" s="12"/>
+    </row>
+    <row r="22" spans="1:11" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A22">
         <v>25</v>
       </c>
-      <c r="I4" s="2" t="s">
-        <v>23</v>
+      <c r="B22" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="C22" s="9" t="s">
+        <v>181</v>
+      </c>
+      <c r="D22" s="1">
+        <v>44378</v>
+      </c>
+      <c r="E22" s="2" t="s">
+        <v>183</v>
+      </c>
+      <c r="F22" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="G22" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="H22" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="I22" s="2" t="s">
+        <v>187</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="172.8" x14ac:dyDescent="0.3">
-      <c r="A5">
-        <v>4</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="C5" s="9" t="s">
-        <v>29</v>
-      </c>
-      <c r="D5" s="1">
-        <v>45778</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="F5" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="G5" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="H5" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="I5" s="2" t="s">
-        <v>34</v>
+    <row r="23" spans="1:11" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A23">
+        <v>11</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="C23" s="9" t="s">
+        <v>85</v>
+      </c>
+      <c r="D23" s="1">
+        <v>44228</v>
+      </c>
+      <c r="E23" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="F23" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="G23" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="H23" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="I23" s="2" t="s">
+        <v>90</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="331.2" x14ac:dyDescent="0.3">
-      <c r="A6">
+    <row r="24" spans="1:11" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A24">
         <v>5</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B24" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="C6" s="9" t="s">
+      <c r="C24" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="D6" s="1">
+      <c r="D24" s="1">
         <v>44136</v>
       </c>
-      <c r="E6" s="2" t="s">
+      <c r="E24" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="F6" s="4" t="s">
+      <c r="F24" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="G6" s="2" t="s">
+      <c r="G24" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="H6" s="4" t="s">
+      <c r="H24" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="I6" s="4" t="s">
+      <c r="I24" s="4" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="409.6" x14ac:dyDescent="0.3">
-      <c r="A7">
-        <v>6</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="C7" s="9" t="s">
-        <v>45</v>
-      </c>
-      <c r="D7" s="10">
-        <v>45047</v>
-      </c>
-      <c r="E7" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="F7" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="G7" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="H7" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="I7" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="J7" s="2" t="s">
-        <v>52</v>
+    <row r="25" spans="1:11" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A25">
+        <v>26</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="C25" s="9" t="s">
+        <v>188</v>
+      </c>
+      <c r="D25" s="1">
+        <v>43925</v>
+      </c>
+      <c r="E25" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="F25" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="G25" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="H25" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="I25" s="2" t="s">
+        <v>194</v>
       </c>
     </row>
-    <row r="8" spans="1:11" ht="409.6" x14ac:dyDescent="0.3">
-      <c r="A8">
-        <v>7</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="C8" s="9" t="s">
-        <v>54</v>
-      </c>
-      <c r="D8" s="1">
-        <v>45505</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="F8" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="G8" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="H8" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="I8" s="2" t="s">
-        <v>59</v>
+    <row r="26" spans="1:11" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A26">
+        <v>10</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="C26" s="9" t="s">
+        <v>78</v>
+      </c>
+      <c r="D26" s="1">
+        <v>43922</v>
+      </c>
+      <c r="E26" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="F26" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="G26" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="H26" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="I26" s="2" t="s">
+        <v>83</v>
       </c>
     </row>
-    <row r="9" spans="1:11" ht="409.6" x14ac:dyDescent="0.3">
-      <c r="A9">
+    <row r="27" spans="1:11" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A27">
         <v>8</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B27" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="C9" s="9" t="s">
+      <c r="C27" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="D9" s="1">
+      <c r="D27" s="1">
         <v>43709</v>
       </c>
-      <c r="E9" s="2" t="s">
+      <c r="E27" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="F9" s="2" t="s">
+      <c r="F27" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="G9" s="2" t="s">
+      <c r="G27" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="H9" s="2" t="s">
+      <c r="H27" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="I9" s="2" t="s">
+      <c r="I27" s="2" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="10" spans="1:11" ht="409.6" x14ac:dyDescent="0.3">
-      <c r="A10">
+    <row r="28" spans="1:11" s="12" customFormat="1" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A28">
         <v>9</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B28" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="C10" s="9" t="s">
+      <c r="C28" s="9" t="s">
         <v>68</v>
       </c>
-      <c r="D10" s="10">
+      <c r="D28" s="10">
         <v>43435</v>
       </c>
-      <c r="E10" s="2" t="s">
+      <c r="E28" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="F10" s="2" t="s">
+      <c r="F28" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="G10" s="2" t="s">
+      <c r="G28" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="H10" s="2" t="s">
+      <c r="H28" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="I10" s="2" t="s">
+      <c r="I28" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="J10" s="2" t="s">
+      <c r="J28" s="2" t="s">
         <v>73</v>
       </c>
+      <c r="K28"/>
     </row>
-    <row r="11" spans="1:11" ht="409.6" x14ac:dyDescent="0.3">
-      <c r="A11">
-        <v>10</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="C11" s="9" t="s">
-        <v>78</v>
-      </c>
-      <c r="D11" s="1">
-        <v>43922</v>
-      </c>
-      <c r="E11" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="F11" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="G11" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="H11" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="I11" s="2" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" ht="409.6" x14ac:dyDescent="0.3">
-      <c r="A12">
-        <v>11</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="C12" s="9" t="s">
-        <v>85</v>
-      </c>
-      <c r="D12" s="1">
-        <v>44228</v>
-      </c>
-      <c r="E12" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="F12" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="G12" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="H12" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="I12" s="2" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
         <v>91</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11" ht="403.2" x14ac:dyDescent="0.3">
-      <c r="A14">
-        <v>13</v>
-      </c>
-      <c r="B14" t="s">
-        <v>92</v>
-      </c>
-      <c r="C14" s="9" t="s">
-        <v>93</v>
-      </c>
-      <c r="D14" s="1">
-        <v>44743</v>
-      </c>
-      <c r="E14" s="2" t="s">
-        <v>94</v>
-      </c>
-      <c r="F14" s="2" t="s">
-        <v>95</v>
-      </c>
-      <c r="G14" s="2" t="s">
-        <v>96</v>
-      </c>
-      <c r="H14" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="I14" s="2" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="15" spans="1:11" ht="360" x14ac:dyDescent="0.3">
-      <c r="A15">
-        <v>14</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>100</v>
-      </c>
-      <c r="C15" s="9" t="s">
-        <v>99</v>
-      </c>
-      <c r="D15" s="1">
-        <v>45748</v>
-      </c>
-      <c r="E15" s="2" t="s">
-        <v>101</v>
-      </c>
-      <c r="F15" s="2" t="s">
-        <v>102</v>
-      </c>
-      <c r="G15" s="2" t="s">
-        <v>103</v>
-      </c>
-      <c r="H15" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="I15" s="2" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="16" spans="1:11" s="12" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
-      <c r="A16" s="12">
-        <v>15</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="C16" s="13" t="s">
-        <v>107</v>
-      </c>
-      <c r="D16" s="14">
-        <v>45078</v>
-      </c>
-      <c r="E16" s="15" t="s">
-        <v>108</v>
-      </c>
-      <c r="F16" s="16" t="s">
-        <v>109</v>
-      </c>
-      <c r="G16" s="16" t="s">
-        <v>110</v>
-      </c>
-      <c r="H16" s="16" t="s">
-        <v>111</v>
-      </c>
-      <c r="I16" s="16" t="s">
-        <v>114</v>
-      </c>
-      <c r="J16" s="16" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="17" spans="1:9" ht="360" x14ac:dyDescent="0.3">
-      <c r="A17">
-        <v>16</v>
-      </c>
-      <c r="B17" s="2" t="s">
-        <v>115</v>
-      </c>
-      <c r="C17" s="9" t="s">
-        <v>116</v>
-      </c>
-      <c r="D17" s="1">
-        <v>44593</v>
-      </c>
-      <c r="E17" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="F17" s="2" t="s">
-        <v>118</v>
-      </c>
-      <c r="G17" s="2" t="s">
-        <v>119</v>
-      </c>
-      <c r="H17" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="I17" s="2" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="18" spans="1:9" ht="409.6" x14ac:dyDescent="0.3">
-      <c r="A18">
-        <v>17</v>
-      </c>
-      <c r="B18" s="2" t="s">
-        <v>122</v>
-      </c>
-      <c r="C18" s="9" t="s">
-        <v>123</v>
-      </c>
-      <c r="D18" s="1">
-        <v>45748</v>
-      </c>
-      <c r="E18" s="11" t="s">
-        <v>124</v>
-      </c>
-      <c r="F18" s="11" t="s">
-        <v>125</v>
-      </c>
-      <c r="G18" s="2" t="s">
-        <v>127</v>
-      </c>
-      <c r="H18" s="2" t="s">
-        <v>128</v>
-      </c>
-      <c r="I18" s="2" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="19" spans="1:9" ht="374.4" x14ac:dyDescent="0.3">
-      <c r="A19">
-        <v>18</v>
-      </c>
-      <c r="B19" s="2" t="s">
-        <v>130</v>
-      </c>
-      <c r="C19" s="9" t="s">
-        <v>131</v>
-      </c>
-      <c r="D19" s="1">
-        <v>45047</v>
-      </c>
-      <c r="E19" s="11" t="s">
-        <v>132</v>
-      </c>
-      <c r="F19" s="11" t="s">
-        <v>133</v>
-      </c>
-      <c r="G19" s="2" t="s">
-        <v>134</v>
-      </c>
-      <c r="H19" s="11" t="s">
-        <v>135</v>
-      </c>
-      <c r="I19" s="11" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="20" spans="1:9" s="12" customFormat="1" ht="331.2" x14ac:dyDescent="0.3">
-      <c r="A20" s="12">
-        <v>19</v>
-      </c>
-      <c r="B20" s="16" t="s">
-        <v>137</v>
-      </c>
-      <c r="C20" s="13" t="s">
-        <v>138</v>
-      </c>
-      <c r="D20" s="14">
-        <v>45505</v>
-      </c>
-      <c r="E20" s="15" t="s">
-        <v>139</v>
-      </c>
-      <c r="F20" s="16" t="s">
-        <v>140</v>
-      </c>
-      <c r="G20" s="16" t="s">
-        <v>141</v>
-      </c>
-      <c r="H20" s="16" t="s">
-        <v>142</v>
-      </c>
-      <c r="I20" s="16" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="21" spans="1:9" ht="403.2" x14ac:dyDescent="0.3">
-      <c r="A21">
-        <v>20</v>
-      </c>
-      <c r="B21" s="2" t="s">
-        <v>145</v>
-      </c>
-      <c r="C21" s="2" t="s">
-        <v>144</v>
-      </c>
-      <c r="D21" s="1">
-        <v>45352</v>
-      </c>
-      <c r="E21" s="11" t="s">
-        <v>146</v>
-      </c>
-      <c r="F21" s="11" t="s">
-        <v>147</v>
-      </c>
-      <c r="G21" s="2" t="s">
-        <v>148</v>
-      </c>
-      <c r="H21" s="2" t="s">
-        <v>149</v>
-      </c>
-      <c r="I21" s="2" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="22" spans="1:9" ht="388.8" x14ac:dyDescent="0.3">
-      <c r="A22">
-        <v>21</v>
-      </c>
-      <c r="B22" s="2" t="s">
-        <v>151</v>
-      </c>
-      <c r="C22" s="9" t="s">
-        <v>152</v>
-      </c>
-      <c r="D22" s="1">
-        <v>45383</v>
-      </c>
-      <c r="E22" s="11" t="s">
-        <v>153</v>
-      </c>
-      <c r="F22" s="2" t="s">
-        <v>154</v>
-      </c>
-      <c r="G22" s="2" t="s">
-        <v>155</v>
-      </c>
-      <c r="H22" s="2" t="s">
-        <v>156</v>
-      </c>
-      <c r="I22" s="2" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="23" spans="1:9" ht="409.6" x14ac:dyDescent="0.3">
-      <c r="A23">
-        <v>22</v>
-      </c>
-      <c r="B23" s="2" t="s">
-        <v>158</v>
-      </c>
-      <c r="C23" s="9" t="s">
-        <v>159</v>
-      </c>
-      <c r="D23" s="1">
-        <v>45261</v>
-      </c>
-      <c r="E23" s="2" t="s">
-        <v>160</v>
-      </c>
-      <c r="F23" s="2" t="s">
-        <v>161</v>
-      </c>
-      <c r="G23" s="2" t="s">
-        <v>162</v>
-      </c>
-      <c r="H23" s="2" t="s">
-        <v>163</v>
-      </c>
-      <c r="I23" s="2" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="24" spans="1:9" ht="409.6" x14ac:dyDescent="0.3">
-      <c r="A24">
-        <v>23</v>
-      </c>
-      <c r="B24" s="2" t="s">
-        <v>166</v>
-      </c>
-      <c r="C24" s="9" t="s">
-        <v>165</v>
-      </c>
-      <c r="D24" s="1">
-        <v>45078</v>
-      </c>
-      <c r="E24" s="2" t="s">
-        <v>167</v>
-      </c>
-      <c r="F24" s="2" t="s">
-        <v>168</v>
-      </c>
-      <c r="G24" s="2" t="s">
-        <v>169</v>
-      </c>
-      <c r="H24" s="2" t="s">
-        <v>170</v>
-      </c>
-      <c r="I24" s="2" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="25" spans="1:9" ht="409.6" x14ac:dyDescent="0.3">
-      <c r="A25">
-        <v>24</v>
-      </c>
-      <c r="B25" s="2" t="s">
-        <v>173</v>
-      </c>
-      <c r="C25" s="9" t="s">
-        <v>172</v>
-      </c>
-      <c r="D25" s="1">
-        <v>44958</v>
-      </c>
-      <c r="E25" s="2" t="s">
-        <v>174</v>
-      </c>
-      <c r="F25" s="2" t="s">
-        <v>177</v>
-      </c>
-      <c r="G25" s="2" t="s">
-        <v>178</v>
-      </c>
-      <c r="H25" s="2" t="s">
-        <v>179</v>
-      </c>
-      <c r="I25" s="2" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="26" spans="1:9" ht="409.6" x14ac:dyDescent="0.3">
-      <c r="A26">
-        <v>25</v>
-      </c>
-      <c r="B26" s="2" t="s">
-        <v>182</v>
-      </c>
-      <c r="C26" s="9" t="s">
-        <v>181</v>
-      </c>
-      <c r="D26" s="1">
-        <v>44378</v>
-      </c>
-      <c r="E26" s="2" t="s">
-        <v>183</v>
-      </c>
-      <c r="F26" s="2" t="s">
-        <v>184</v>
-      </c>
-      <c r="G26" s="2" t="s">
-        <v>185</v>
-      </c>
-      <c r="H26" s="2" t="s">
-        <v>186</v>
-      </c>
-      <c r="I26" s="2" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="27" spans="1:9" ht="409.6" x14ac:dyDescent="0.3">
-      <c r="A27">
-        <v>26</v>
-      </c>
-      <c r="B27" s="2" t="s">
-        <v>189</v>
-      </c>
-      <c r="C27" s="9" t="s">
-        <v>188</v>
-      </c>
-      <c r="D27" s="1">
-        <v>43925</v>
-      </c>
-      <c r="E27" s="2" t="s">
-        <v>190</v>
-      </c>
-      <c r="F27" s="2" t="s">
-        <v>191</v>
-      </c>
-      <c r="G27" s="2" t="s">
-        <v>192</v>
-      </c>
-      <c r="H27" s="2" t="s">
-        <v>193</v>
-      </c>
-      <c r="I27" s="2" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="28" spans="1:9" s="12" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
-      <c r="A28" s="12">
-        <v>27</v>
-      </c>
-      <c r="B28" s="16" t="s">
-        <v>195</v>
-      </c>
-      <c r="C28" s="13" t="s">
-        <v>93</v>
-      </c>
-      <c r="D28" s="14">
-        <v>44470</v>
-      </c>
-      <c r="E28" s="16" t="s">
-        <v>196</v>
-      </c>
-      <c r="F28" s="16" t="s">
-        <v>197</v>
-      </c>
-      <c r="G28" s="16" t="s">
-        <v>198</v>
-      </c>
-      <c r="H28" s="16" t="s">
-        <v>199</v>
-      </c>
-      <c r="I28" s="16" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="29" spans="1:9" ht="409.6" x14ac:dyDescent="0.3">
-      <c r="A29">
-        <v>28</v>
-      </c>
-      <c r="B29" s="2" t="s">
-        <v>202</v>
-      </c>
-      <c r="C29" s="9" t="s">
-        <v>201</v>
-      </c>
-      <c r="D29" s="1">
-        <v>45292</v>
-      </c>
-      <c r="E29" s="2" t="s">
-        <v>203</v>
-      </c>
-      <c r="F29" s="2" t="s">
-        <v>204</v>
-      </c>
-      <c r="G29" s="2" t="s">
-        <v>205</v>
-      </c>
-      <c r="H29" s="2" t="s">
-        <v>206</v>
-      </c>
-      <c r="I29" s="2" t="s">
-        <v>207</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:K1" xr:uid="{E3273017-25D8-4705-B64D-E4EEBFC32101}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:K30">
+    <sortCondition descending="1" ref="D1:D30"/>
+  </sortState>
   <hyperlinks>
-    <hyperlink ref="C5" r:id="rId1" display="https://papers.ssrn.com/sol3/papers.cfm?abstract_id=5259722" xr:uid="{F6709356-ED4B-4A5B-BFD4-4B669ED87300}"/>
-    <hyperlink ref="C6" r:id="rId2" display="https://aclanthology.org/2020.privatenlp-1.5/" xr:uid="{E91A3E06-C7C0-4232-9B9C-958A53660944}"/>
-    <hyperlink ref="C7" r:id="rId3" display="https://arxiv.org/abs/2305.18396" xr:uid="{89A300C5-1B74-446C-9D44-77A7BAE19972}"/>
-    <hyperlink ref="C8" r:id="rId4" display="https://arxiv.org/abs/2310.09130" xr:uid="{D265B287-0711-4975-B3DA-D46D676E79F2}"/>
-    <hyperlink ref="C9" r:id="rId5" display="https://arxiv.org/abs/1909.09145" xr:uid="{E6F068DA-77A1-4AF2-BCB8-BAB1BC5F99D5}"/>
-    <hyperlink ref="C10" r:id="rId6" display="https://arxiv.org/abs/1812.00564" xr:uid="{991C14EA-F987-461D-BB97-BBF6D1AC7EB3}"/>
-    <hyperlink ref="C11" r:id="rId7" display="https://ieeexplore.ieee.org/document/9069945" xr:uid="{9383D204-9E86-40EF-B6EF-4CF1D0575D5D}"/>
-    <hyperlink ref="C12" r:id="rId8" display="https://arxiv.org/abs/2102.08504" xr:uid="{237D23DB-0320-4B06-979D-E8C5F5641137}"/>
-    <hyperlink ref="C14" r:id="rId9" display="https://arxiv.org/abs/2110.06500" xr:uid="{593B325C-8AB0-44E3-B5C4-EBAD0E85E02F}"/>
-    <hyperlink ref="C15" r:id="rId10" display="https://dl.acm.org/doi/abs/10.1145/3696410.3714531" xr:uid="{D2AD492D-EBD8-437E-B49F-4D74653F8A2E}"/>
-    <hyperlink ref="C16" r:id="rId11" display="https://arxiv.org/abs/2306.08223" xr:uid="{A7C8098E-424D-4A84-A80E-7643C924F821}"/>
-    <hyperlink ref="C17" r:id="rId12" display="https://arxiv.org/abs/2202.05520" xr:uid="{2AFA1272-530E-472C-AA98-4FAB1E668DD0}"/>
-    <hyperlink ref="C18" r:id="rId13" display="https://dl.acm.org/doi/full/10.1145/3706598.3713701" xr:uid="{FA079AEC-4E31-444F-B03C-FEF634B1EBC1}"/>
-    <hyperlink ref="C19" r:id="rId14" display="https://arxiv.org/abs/2305.15008" xr:uid="{2E5787C8-6AA0-4059-8C31-659EF5D13331}"/>
-    <hyperlink ref="C20" r:id="rId15" display="https://arxiv.org/abs/2408.07004" xr:uid="{9A475C34-F3D2-4BD8-900A-086E09E58594}"/>
-    <hyperlink ref="C22" r:id="rId16" display="https://ieeexplore.ieee.org/document/10447454" xr:uid="{6B4D055D-5DA2-4ADC-B931-B85BCE8326AA}"/>
-    <hyperlink ref="C23" r:id="rId17" display="https://aclanthology.org/2023.emnlp-main.921/" xr:uid="{CBC3D013-B497-49AA-A3BF-10F361C07017}"/>
-    <hyperlink ref="C24" r:id="rId18" display="https://aclanthology.org/2023.inlg-main.3/" xr:uid="{2C70D679-6874-4A32-B394-DE8078918BC2}"/>
-    <hyperlink ref="B24" r:id="rId19" display="https://aclanthology.org/2023.inlg-main.3.pdf" xr:uid="{96A42630-64DF-445C-9AA6-EAF5C8EF714C}"/>
-    <hyperlink ref="C25" r:id="rId20" display="https://arxiv.org/abs/2302.00539" xr:uid="{D9A12C70-0468-4FB5-B9B9-48850E614F95}"/>
-    <hyperlink ref="C26" r:id="rId21" display="https://arxiv.org/abs/2107.01614" xr:uid="{B311B9FF-1E74-4350-BB2E-9F8452AD7C69}"/>
-    <hyperlink ref="C27" r:id="rId22" display="https://pubmed.ncbi.nlm.nih.gov/34350426/" xr:uid="{D434CFB1-40DD-4122-8E69-F7F6EA3277F0}"/>
-    <hyperlink ref="C28" r:id="rId23" display="https://arxiv.org/abs/2110.06500" xr:uid="{BEE0DB7E-EE1A-4795-ACF9-5E7286358DC8}"/>
-    <hyperlink ref="C29" r:id="rId24" display="https://www.academia.edu/124958504/Navigating_Data_Protection_Challenges_in_the_Era_of_Artificial_Intelligence_A_Comprehensive_Review" xr:uid="{40E33EEC-6A75-4617-BE2D-ED27CBBF739A}"/>
+    <hyperlink ref="C3" r:id="rId1" display="https://papers.ssrn.com/sol3/papers.cfm?abstract_id=5259722" xr:uid="{F6709356-ED4B-4A5B-BFD4-4B669ED87300}"/>
+    <hyperlink ref="C24" r:id="rId2" display="https://aclanthology.org/2020.privatenlp-1.5/" xr:uid="{E91A3E06-C7C0-4232-9B9C-958A53660944}"/>
+    <hyperlink ref="C16" r:id="rId3" display="https://arxiv.org/abs/2305.18396" xr:uid="{89A300C5-1B74-446C-9D44-77A7BAE19972}"/>
+    <hyperlink ref="C6" r:id="rId4" display="https://arxiv.org/abs/2310.09130" xr:uid="{D265B287-0711-4975-B3DA-D46D676E79F2}"/>
+    <hyperlink ref="C27" r:id="rId5" display="https://arxiv.org/abs/1909.09145" xr:uid="{E6F068DA-77A1-4AF2-BCB8-BAB1BC5F99D5}"/>
+    <hyperlink ref="C28" r:id="rId6" display="https://arxiv.org/abs/1812.00564" xr:uid="{991C14EA-F987-461D-BB97-BBF6D1AC7EB3}"/>
+    <hyperlink ref="C26" r:id="rId7" display="https://ieeexplore.ieee.org/document/9069945" xr:uid="{9383D204-9E86-40EF-B6EF-4CF1D0575D5D}"/>
+    <hyperlink ref="C23" r:id="rId8" display="https://arxiv.org/abs/2102.08504" xr:uid="{237D23DB-0320-4B06-979D-E8C5F5641137}"/>
+    <hyperlink ref="C19" r:id="rId9" display="https://arxiv.org/abs/2110.06500" xr:uid="{593B325C-8AB0-44E3-B5C4-EBAD0E85E02F}"/>
+    <hyperlink ref="C4" r:id="rId10" display="https://dl.acm.org/doi/abs/10.1145/3696410.3714531" xr:uid="{D2AD492D-EBD8-437E-B49F-4D74653F8A2E}"/>
+    <hyperlink ref="C14" r:id="rId11" display="https://arxiv.org/abs/2306.08223" xr:uid="{A7C8098E-424D-4A84-A80E-7643C924F821}"/>
+    <hyperlink ref="C20" r:id="rId12" display="https://arxiv.org/abs/2202.05520" xr:uid="{2AFA1272-530E-472C-AA98-4FAB1E668DD0}"/>
+    <hyperlink ref="C5" r:id="rId13" display="https://dl.acm.org/doi/full/10.1145/3706598.3713701" xr:uid="{FA079AEC-4E31-444F-B03C-FEF634B1EBC1}"/>
+    <hyperlink ref="C17" r:id="rId14" display="https://arxiv.org/abs/2305.15008" xr:uid="{2E5787C8-6AA0-4059-8C31-659EF5D13331}"/>
+    <hyperlink ref="C7" r:id="rId15" display="https://arxiv.org/abs/2408.07004" xr:uid="{9A475C34-F3D2-4BD8-900A-086E09E58594}"/>
+    <hyperlink ref="C8" r:id="rId16" display="https://ieeexplore.ieee.org/document/10447454" xr:uid="{6B4D055D-5DA2-4ADC-B931-B85BCE8326AA}"/>
+    <hyperlink ref="C11" r:id="rId17" display="https://aclanthology.org/2023.emnlp-main.921/" xr:uid="{CBC3D013-B497-49AA-A3BF-10F361C07017}"/>
+    <hyperlink ref="C15" r:id="rId18" display="https://aclanthology.org/2023.inlg-main.3/" xr:uid="{2C70D679-6874-4A32-B394-DE8078918BC2}"/>
+    <hyperlink ref="B15" r:id="rId19" display="https://aclanthology.org/2023.inlg-main.3.pdf" xr:uid="{96A42630-64DF-445C-9AA6-EAF5C8EF714C}"/>
+    <hyperlink ref="C18" r:id="rId20" display="https://arxiv.org/abs/2302.00539" xr:uid="{D9A12C70-0468-4FB5-B9B9-48850E614F95}"/>
+    <hyperlink ref="C22" r:id="rId21" display="https://arxiv.org/abs/2107.01614" xr:uid="{B311B9FF-1E74-4350-BB2E-9F8452AD7C69}"/>
+    <hyperlink ref="C25" r:id="rId22" display="https://pubmed.ncbi.nlm.nih.gov/34350426/" xr:uid="{D434CFB1-40DD-4122-8E69-F7F6EA3277F0}"/>
+    <hyperlink ref="C21" r:id="rId23" display="https://arxiv.org/abs/2110.06500" xr:uid="{BEE0DB7E-EE1A-4795-ACF9-5E7286358DC8}"/>
+    <hyperlink ref="C10" r:id="rId24" display="https://www.academia.edu/124958504/Navigating_Data_Protection_Challenges_in_the_Era_of_Artificial_Intelligence_A_Comprehensive_Review" xr:uid="{40E33EEC-6A75-4617-BE2D-ED27CBBF739A}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -5441,42 +5450,42 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B8FDB45-EE13-4E63-A03A-A7B6283EA313}">
   <dimension ref="B1:D11"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="78.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="78.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B1" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="2" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B2" s="8" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B3" s="8" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="9" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="10" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="11" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
         <v>113</v>
       </c>

</xml_diff>